<commit_message>
docs(pruebas): completa las pruebas de control pendientes de las iteraciones 3 y 5
Se ejecutaron en el entorno QA la reversion de proceso y el balance de masa al finalizar
(Req 003) y la verificacion de las tablas de datos de las graficas en escritorio, tableta y
telefono (Req 005). Ambas hojas quedan con 100 % de pruebas realizadas y exitosas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/pruebas/Resultados_Pruebas_Iteraciones_3_4_5.xlsx
+++ b/docs/pruebas/Resultados_Pruebas_Iteraciones_3_4_5.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B335AF06-AE9F-48B6-9D2B-4BEC3A49AC02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3745A902-DA21-4226-89E7-4B88A6C81911}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Req 003 - Produccion" sheetId="1" r:id="rId1"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="82">
   <si>
     <t>Resultados de Pruebas de Requerimientos Funcionales</t>
   </si>
@@ -212,15 +212,6 @@
     <t>El proceso se marca inactivo y el sub-lote de origen regresa a "Listo para produccion" con el peso restaurado.</t>
   </si>
   <si>
-    <t>NO</t>
-  </si>
-  <si>
-    <t>PENDIENTE</t>
-  </si>
-  <si>
-    <t>Implementado y validado por revision de codigo; pendiente ejecutar prueba en vivo contra la base de datos.</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b/>
@@ -253,9 +244,6 @@
     <t>% Pruebas Realizadas</t>
   </si>
   <si>
-    <t>67%</t>
-  </si>
-  <si>
     <t>% Pruebas Exitosas</t>
   </si>
   <si>
@@ -551,13 +539,19 @@
     <t>La tabla refleja los mismos valores que la grafica y se visualiza correctamente en distintos tamanos de pantalla.</t>
   </si>
   <si>
-    <t>Pendiente verificacion visual en navegador (ajustes de estilo movil en curso).</t>
-  </si>
-  <si>
     <t>Modulo de Reporteria: Graficas del Dashboard (Iteracion 5)</t>
   </si>
   <si>
-    <t>80%</t>
+    <t>22/10/2026</t>
+  </si>
+  <si>
+    <t>Ejecutada en vivo: PRO-000016 revertido; el sub-lote volvio a Listo para produccion con sus 100 kg.</t>
+  </si>
+  <si>
+    <t>Ejecutada en vivo: diferencia de 5 kg rechazada sin justificacion; aceptada al justificarla.</t>
+  </si>
+  <si>
+    <t>Verificada en escritorio, tableta y telefono: cada grafica muestra su tabla legible.</t>
   </si>
 </sst>
 </file>
@@ -629,7 +623,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -661,6 +655,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1237,51 +1237,51 @@
         <v>20</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>27</v>
+        <v>78</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>38</v>
+        <v>79</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="10"/>
       <c r="B13" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>27</v>
+        <v>78</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>38</v>
+        <v>80</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
@@ -1294,7 +1294,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
@@ -1318,26 +1318,26 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B19" s="5"/>
-      <c r="C19" s="6" t="s">
-        <v>44</v>
+      <c r="C19" s="12">
+        <v>1</v>
       </c>
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
       <c r="F19" s="6"/>
       <c r="G19" s="5" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H19" s="5"/>
-      <c r="I19" s="4" t="s">
-        <v>44</v>
+      <c r="I19" s="13">
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="6">
@@ -1349,36 +1349,36 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="6">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D22" s="6"/>
       <c r="E22" s="6"/>
       <c r="F22" s="6"/>
       <c r="G22" s="5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H22" s="5"/>
       <c r="I22" s="4">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D23" s="6"/>
       <c r="E23" s="6"/>
       <c r="F23" s="6"/>
       <c r="G23" s="5" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="H23" s="5"/>
       <c r="I23" s="4">
@@ -1412,7 +1412,7 @@
     <mergeCell ref="G22:H22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1534,13 +1534,13 @@
     </row>
     <row r="8" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>20</v>
@@ -1555,7 +1555,7 @@
         <v>22</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>21</v>
@@ -1564,10 +1564,10 @@
     <row r="9" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="10"/>
       <c r="B9" s="2" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>26</v>
@@ -1591,10 +1591,10 @@
     <row r="10" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="10"/>
       <c r="B10" s="2" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>20</v>
@@ -1618,13 +1618,13 @@
     <row r="11" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="10"/>
       <c r="B11" s="2" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>7</v>
@@ -1645,10 +1645,10 @@
     <row r="12" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="10"/>
       <c r="B12" s="2" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>20</v>
@@ -1672,13 +1672,13 @@
     <row r="13" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="10"/>
       <c r="B13" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>7</v>
@@ -1690,7 +1690,7 @@
         <v>22</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="I13" s="3" t="s">
         <v>21</v>
@@ -1698,7 +1698,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
@@ -1711,7 +1711,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
@@ -1735,26 +1735,26 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="6" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
       <c r="F19" s="6"/>
       <c r="G19" s="5" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H19" s="5"/>
       <c r="I19" s="4" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="6">
@@ -1766,7 +1766,7 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="6">
@@ -1776,7 +1776,7 @@
       <c r="E22" s="6"/>
       <c r="F22" s="6"/>
       <c r="G22" s="5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H22" s="5"/>
       <c r="I22" s="4">
@@ -1785,7 +1785,7 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="6">
@@ -1795,7 +1795,7 @@
       <c r="E23" s="6"/>
       <c r="F23" s="6"/>
       <c r="G23" s="5" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="H23" s="5"/>
       <c r="I23" s="4">
@@ -1951,13 +1951,13 @@
     </row>
     <row r="8" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>26</v>
@@ -1972,7 +1972,7 @@
         <v>22</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>21</v>
@@ -1981,10 +1981,10 @@
     <row r="9" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="10"/>
       <c r="B9" s="2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>26</v>
@@ -2008,10 +2008,10 @@
     <row r="10" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="10"/>
       <c r="B10" s="2" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>26</v>
@@ -2035,10 +2035,10 @@
     <row r="11" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="10"/>
       <c r="B11" s="2" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>26</v>
@@ -2062,33 +2062,33 @@
     <row r="12" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="10"/>
       <c r="B12" s="2" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>26</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>27</v>
+        <v>78</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>81</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
@@ -2101,7 +2101,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -2125,26 +2125,26 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B18" s="5"/>
-      <c r="C18" s="6" t="s">
-        <v>83</v>
+      <c r="C18" s="12">
+        <v>1</v>
       </c>
       <c r="D18" s="6"/>
       <c r="E18" s="6"/>
       <c r="F18" s="6"/>
       <c r="G18" s="5" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H18" s="5"/>
-      <c r="I18" s="4" t="s">
-        <v>83</v>
+      <c r="I18" s="13">
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B20" s="5"/>
       <c r="C20" s="6">
@@ -2156,36 +2156,36 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D21" s="6"/>
       <c r="E21" s="6"/>
       <c r="F21" s="6"/>
       <c r="G21" s="5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H21" s="5"/>
       <c r="I21" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D22" s="6"/>
       <c r="E22" s="6"/>
       <c r="F22" s="6"/>
       <c r="G22" s="5" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="H22" s="5"/>
       <c r="I22" s="4">
@@ -2219,6 +2219,6 @@
     <mergeCell ref="G21:H21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>